<commit_message>
RPA datasets push 2024-08-11
</commit_message>
<xml_diff>
--- a/datasets/form1.xlsx
+++ b/datasets/form1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="92">
   <si>
     <t>상장일</t>
   </si>
@@ -118,162 +118,153 @@
     <t>2024-06-19</t>
   </si>
   <si>
+    <t>2024-07-01</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>SK증권제13호스팩</t>
+  </si>
+  <si>
+    <t>엑셀세라퓨틱스</t>
+  </si>
+  <si>
+    <t>시프트업</t>
+  </si>
+  <si>
+    <t>이베스트스팩6호</t>
+  </si>
+  <si>
+    <t>하스</t>
+  </si>
+  <si>
+    <t>이노스페이스</t>
+  </si>
+  <si>
+    <t>에이치브이엠</t>
+  </si>
+  <si>
+    <t>하이젠알앤엠</t>
+  </si>
+  <si>
+    <t>한국제15호스팩</t>
+  </si>
+  <si>
+    <t>에스오에스랩</t>
+  </si>
+  <si>
+    <t>미래에셋비전스팩6호</t>
+  </si>
+  <si>
+    <t>KB제29호스팩</t>
+  </si>
+  <si>
+    <t>에이치엠씨제7호스팩</t>
+  </si>
+  <si>
+    <t>한국제14호스팩</t>
+  </si>
+  <si>
+    <t>미래에셋비전스팩5호</t>
+  </si>
+  <si>
+    <t>씨어스테크놀로지</t>
+  </si>
+  <si>
+    <t>한중엔시에스</t>
+  </si>
+  <si>
+    <t>신한글로벌액티브리츠</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>제이피모간회사</t>
+  </si>
+  <si>
+    <t>신한</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>BNK</t>
+  </si>
+  <si>
+    <t>KB</t>
+  </si>
+  <si>
+    <t>현대차</t>
+  </si>
+  <si>
+    <t>IBK</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>공동대표</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>2024-07-18</t>
+  </si>
+  <si>
+    <t>2024-07-16</t>
+  </si>
+  <si>
+    <t>2024-06-20</t>
+  </si>
+  <si>
+    <t>2024-06-18</t>
+  </si>
+  <si>
     <t>2024-06-17</t>
   </si>
   <si>
-    <t>2024-06-18</t>
-  </si>
-  <si>
-    <t>2024-07-01</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
-    <t>시프트업</t>
-  </si>
-  <si>
-    <t>이베스트스팩6호</t>
-  </si>
-  <si>
-    <t>하스</t>
-  </si>
-  <si>
-    <t>이노스페이스</t>
-  </si>
-  <si>
-    <t>에이치브이엠</t>
-  </si>
-  <si>
-    <t>하이젠알앤엠</t>
-  </si>
-  <si>
-    <t>한국제15호스팩</t>
-  </si>
-  <si>
-    <t>에스오에스랩</t>
-  </si>
-  <si>
-    <t>미래에셋비전스팩6호</t>
-  </si>
-  <si>
-    <t>KB제29호스팩</t>
-  </si>
-  <si>
-    <t>에이치엠씨제7호스팩</t>
-  </si>
-  <si>
-    <t>한국제14호스팩</t>
-  </si>
-  <si>
-    <t>미래에셋비전스팩5호</t>
-  </si>
-  <si>
-    <t>씨어스테크놀로지</t>
-  </si>
-  <si>
-    <t>한중엔시에스</t>
-  </si>
-  <si>
-    <t>라메디텍</t>
-  </si>
-  <si>
-    <t>디비금융스팩12호</t>
-  </si>
-  <si>
-    <t>신한글로벌액티브리츠</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>제이피모간회사</t>
-  </si>
-  <si>
-    <t>신한</t>
-  </si>
-  <si>
-    <t>LS</t>
-  </si>
-  <si>
-    <t>BNK</t>
-  </si>
-  <si>
-    <t>KB</t>
-  </si>
-  <si>
-    <t>현대차</t>
-  </si>
-  <si>
-    <t>IBK</t>
-  </si>
-  <si>
-    <t>DB</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>공동대표</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
-    <t>2024-06-20</t>
-  </si>
-  <si>
     <t>2024-06-14</t>
   </si>
   <si>
@@ -284,9 +275,6 @@
   </si>
   <si>
     <t>2024-06-10</t>
-  </si>
-  <si>
-    <t>2024-06-05</t>
   </si>
   <si>
     <t>2024-07-30</t>
@@ -659,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -720,37 +708,37 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D2">
         <v>223.4</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F2">
         <v>223.4</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M2">
         <v>10000</v>
@@ -762,7 +750,7 @@
         <v>21</v>
       </c>
       <c r="P2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="Q2">
         <v>1675500</v>
@@ -773,37 +761,37 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D3">
         <v>297</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>297</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M3">
         <v>22000</v>
@@ -812,7 +800,7 @@
         <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="P3" t="s">
         <v>21</v>
@@ -826,37 +814,37 @@
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D4">
         <v>2660</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F4">
         <v>2553.6</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M4">
         <v>35000</v>
@@ -865,10 +853,10 @@
         <v>96</v>
       </c>
       <c r="O4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="P4" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="Q4">
         <v>9340690</v>
@@ -879,37 +867,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D5">
         <v>2660</v>
       </c>
       <c r="E5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F5">
         <v>106.4</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="L5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M5">
         <v>35000</v>
@@ -918,10 +906,10 @@
         <v>4</v>
       </c>
       <c r="O5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="P5" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="Q5">
         <v>9340690</v>
@@ -932,37 +920,37 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D6">
         <v>120</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F6">
         <v>120</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K6" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M6">
         <v>2000</v>
@@ -971,10 +959,10 @@
         <v>100</v>
       </c>
       <c r="O6" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="P6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="Q6">
         <v>4500000</v>
@@ -985,37 +973,37 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D7">
         <v>80</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F7">
         <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K7" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M7">
         <v>2000</v>
@@ -1027,7 +1015,7 @@
         <v>22</v>
       </c>
       <c r="P7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="Q7">
         <v>3000000</v>
@@ -1038,37 +1026,37 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D8">
         <v>161.8</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F8">
         <v>161.8</v>
       </c>
       <c r="G8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K8" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M8">
         <v>10000</v>
@@ -1080,7 +1068,7 @@
         <v>25</v>
       </c>
       <c r="P8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="Q8">
         <v>1187900</v>
@@ -1091,37 +1079,37 @@
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>4350</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F9">
         <v>1435.5</v>
       </c>
       <c r="G9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M9">
         <v>60000</v>
@@ -1133,7 +1121,7 @@
         <v>26</v>
       </c>
       <c r="P9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="Q9">
         <v>21750000</v>
@@ -1144,37 +1132,37 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D10">
         <v>4350</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F10">
         <v>1435.5</v>
       </c>
       <c r="G10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K10" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M10">
         <v>60000</v>
@@ -1186,7 +1174,7 @@
         <v>26</v>
       </c>
       <c r="P10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="Q10">
         <v>21750000</v>
@@ -1197,37 +1185,37 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D11">
         <v>4350</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F11">
         <v>1305</v>
       </c>
       <c r="G11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M11">
         <v>60000</v>
@@ -1239,7 +1227,7 @@
         <v>26</v>
       </c>
       <c r="P11" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="Q11">
         <v>21750000</v>
@@ -1250,37 +1238,37 @@
         <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D12">
         <v>4350</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F12">
         <v>174</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K12" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="L12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M12">
         <v>60000</v>
@@ -1292,7 +1280,7 @@
         <v>26</v>
       </c>
       <c r="P12" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="Q12">
         <v>21750000</v>
@@ -1303,37 +1291,37 @@
         <v>24</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D13">
         <v>80</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F13">
         <v>80</v>
       </c>
       <c r="G13" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H13" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I13" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J13" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K13" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L13" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M13">
         <v>2000</v>
@@ -1345,7 +1333,7 @@
         <v>26</v>
       </c>
       <c r="P13" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="Q13">
         <v>3000000</v>
@@ -1356,37 +1344,37 @@
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D14">
         <v>289.6</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F14">
         <v>289.6</v>
       </c>
       <c r="G14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M14">
         <v>16000</v>
@@ -1409,37 +1397,37 @@
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D15">
         <v>575.89</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F15">
         <v>541.3366</v>
       </c>
       <c r="G15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K15" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M15">
         <v>43300</v>
@@ -1448,7 +1436,7 @@
         <v>94</v>
       </c>
       <c r="O15" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="P15" t="s">
         <v>30</v>
@@ -1462,37 +1450,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D16">
         <v>575.89</v>
       </c>
       <c r="E16" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F16">
         <v>34.5534</v>
       </c>
       <c r="G16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K16" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="L16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M16">
         <v>43300</v>
@@ -1501,7 +1489,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="P16" t="s">
         <v>30</v>
@@ -1515,37 +1503,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D17">
         <v>432</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F17">
         <v>432</v>
       </c>
       <c r="G17" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H17" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I17" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J17" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K17" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L17" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M17">
         <v>18000</v>
@@ -1568,37 +1556,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D18">
         <v>238</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F18">
         <v>238</v>
       </c>
       <c r="G18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K18" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M18">
         <v>7000</v>
@@ -1607,7 +1595,7 @@
         <v>100</v>
       </c>
       <c r="O18" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="P18" t="s">
         <v>32</v>
@@ -1621,37 +1609,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D19">
         <v>125</v>
       </c>
       <c r="E19" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F19">
         <v>125</v>
       </c>
       <c r="G19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K19" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M19">
         <v>2000</v>
@@ -1660,10 +1648,10 @@
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="P19" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="Q19">
         <v>4687500</v>
@@ -1674,37 +1662,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D20">
         <v>230</v>
       </c>
       <c r="E20" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F20">
         <v>218.5</v>
       </c>
       <c r="G20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K20" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M20">
         <v>11500</v>
@@ -1713,7 +1701,7 @@
         <v>95</v>
       </c>
       <c r="O20" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="P20" t="s">
         <v>33</v>
@@ -1727,37 +1715,37 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D21">
         <v>230</v>
       </c>
       <c r="E21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F21">
         <v>11.5</v>
       </c>
       <c r="G21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K21" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="L21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M21">
         <v>11500</v>
@@ -1766,7 +1754,7 @@
         <v>5</v>
       </c>
       <c r="O21" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="P21" t="s">
         <v>33</v>
@@ -1780,37 +1768,37 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D22">
         <v>129</v>
       </c>
       <c r="E22" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F22">
         <v>129</v>
       </c>
       <c r="G22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K22" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M22">
         <v>2000</v>
@@ -1819,10 +1807,10 @@
         <v>100</v>
       </c>
       <c r="O22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P22" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="Q22">
         <v>4837500</v>
@@ -1833,37 +1821,37 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D23">
         <v>120</v>
       </c>
       <c r="E23" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F23">
         <v>120</v>
       </c>
       <c r="G23" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H23" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I23" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J23" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K23" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L23" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M23">
         <v>2000</v>
@@ -1872,10 +1860,10 @@
         <v>100</v>
       </c>
       <c r="O23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="P23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="Q23">
         <v>4500000</v>
@@ -1886,37 +1874,37 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D24">
         <v>140</v>
       </c>
       <c r="E24" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F24">
         <v>140</v>
       </c>
       <c r="G24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K24" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M24">
         <v>2000</v>
@@ -1925,10 +1913,10 @@
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="P24" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="Q24">
         <v>5250000</v>
@@ -1939,37 +1927,37 @@
         <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D25">
         <v>80</v>
       </c>
       <c r="E25" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F25">
         <v>80</v>
       </c>
       <c r="G25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K25" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M25">
         <v>2000</v>
@@ -1978,10 +1966,10 @@
         <v>100</v>
       </c>
       <c r="O25" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P25" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Q25">
         <v>3000000</v>
@@ -1992,37 +1980,37 @@
         <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D26">
         <v>95</v>
       </c>
       <c r="E26" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F26">
         <v>95</v>
       </c>
       <c r="G26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M26">
         <v>2000</v>
@@ -2031,10 +2019,10 @@
         <v>100</v>
       </c>
       <c r="O26" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P26" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Q26">
         <v>3562500</v>
@@ -2045,37 +2033,37 @@
         <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D27">
         <v>221</v>
       </c>
       <c r="E27" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F27">
         <v>221</v>
       </c>
       <c r="G27" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H27" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I27" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J27" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K27" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L27" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M27">
         <v>17000</v>
@@ -2084,10 +2072,10 @@
         <v>100</v>
       </c>
       <c r="O27" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P27" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Q27">
         <v>975000</v>
@@ -2098,37 +2086,37 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" t="s">
         <v>57</v>
-      </c>
-      <c r="C28" t="s">
-        <v>61</v>
       </c>
       <c r="D28">
         <v>480</v>
       </c>
       <c r="E28" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F28">
         <v>480</v>
       </c>
       <c r="G28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K28" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M28">
         <v>30000</v>
@@ -2137,10 +2125,10 @@
         <v>100</v>
       </c>
       <c r="O28" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Q28">
         <v>1123925</v>
@@ -2151,210 +2139,104 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" t="s">
         <v>58</v>
       </c>
-      <c r="C29" t="s">
-        <v>61</v>
-      </c>
       <c r="D29">
-        <v>207.68</v>
+        <v>700.0000199999999</v>
       </c>
       <c r="E29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F29">
-        <v>207.68</v>
+        <v>350.00001</v>
       </c>
       <c r="G29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K29" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M29">
-        <v>16000</v>
+        <v>3000</v>
       </c>
       <c r="N29">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O29" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="P29" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="Q29">
-        <v>957220</v>
+        <v>32666668</v>
       </c>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C30" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D30">
-        <v>100</v>
+        <v>700.0000199999999</v>
       </c>
       <c r="E30" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="F30">
-        <v>100</v>
+        <v>350.00001</v>
       </c>
       <c r="G30" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H30" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="I30" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="J30" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K30" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L30" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M30">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="N30">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O30" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="P30" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="Q30">
-        <v>3750000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17">
-      <c r="A31" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" t="s">
-        <v>60</v>
-      </c>
-      <c r="C31" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31">
-        <v>700.0000199999999</v>
-      </c>
-      <c r="E31" t="s">
-        <v>71</v>
-      </c>
-      <c r="F31">
-        <v>350.00001</v>
-      </c>
-      <c r="G31" t="s">
-        <v>78</v>
-      </c>
-      <c r="H31" t="s">
-        <v>78</v>
-      </c>
-      <c r="I31" t="s">
-        <v>78</v>
-      </c>
-      <c r="J31" t="s">
-        <v>78</v>
-      </c>
-      <c r="K31" t="s">
-        <v>81</v>
-      </c>
-      <c r="L31" t="s">
-        <v>78</v>
-      </c>
-      <c r="M31">
-        <v>3000</v>
-      </c>
-      <c r="N31">
-        <v>50</v>
-      </c>
-      <c r="O31" t="s">
-        <v>87</v>
-      </c>
-      <c r="P31" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q31">
-        <v>32666668</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17">
-      <c r="A32" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" t="s">
-        <v>60</v>
-      </c>
-      <c r="C32" t="s">
-        <v>62</v>
-      </c>
-      <c r="D32">
-        <v>700.0000199999999</v>
-      </c>
-      <c r="E32" t="s">
-        <v>69</v>
-      </c>
-      <c r="F32">
-        <v>350.00001</v>
-      </c>
-      <c r="G32" t="s">
-        <v>78</v>
-      </c>
-      <c r="H32" t="s">
-        <v>78</v>
-      </c>
-      <c r="I32" t="s">
-        <v>78</v>
-      </c>
-      <c r="J32" t="s">
-        <v>78</v>
-      </c>
-      <c r="K32" t="s">
-        <v>81</v>
-      </c>
-      <c r="L32" t="s">
-        <v>78</v>
-      </c>
-      <c r="M32">
-        <v>3000</v>
-      </c>
-      <c r="N32">
-        <v>50</v>
-      </c>
-      <c r="O32" t="s">
-        <v>87</v>
-      </c>
-      <c r="P32" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q32">
         <v>32666668</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-13
</commit_message>
<xml_diff>
--- a/datasets/form1.xlsx
+++ b/datasets/form1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="89">
   <si>
     <t>상장일</t>
   </si>
@@ -67,6 +67,9 @@
     <t>총기관배정수량</t>
   </si>
   <si>
+    <t>2024-08-12</t>
+  </si>
+  <si>
     <t>2024-08-06</t>
   </si>
   <si>
@@ -115,150 +118,141 @@
     <t>2024-06-21</t>
   </si>
   <si>
+    <t>2024-07-01</t>
+  </si>
+  <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
+    <t>아이빔테크놀로지</t>
+  </si>
+  <si>
+    <t>피앤에스미캐닉스</t>
+  </si>
+  <si>
+    <t>산일전기</t>
+  </si>
+  <si>
+    <t>엔에이치스팩31호</t>
+  </si>
+  <si>
+    <t>SK증권제13호스팩</t>
+  </si>
+  <si>
+    <t>엑셀세라퓨틱스</t>
+  </si>
+  <si>
+    <t>시프트업</t>
+  </si>
+  <si>
+    <t>이베스트스팩6호</t>
+  </si>
+  <si>
+    <t>하스</t>
+  </si>
+  <si>
+    <t>이노스페이스</t>
+  </si>
+  <si>
+    <t>에이치브이엠</t>
+  </si>
+  <si>
+    <t>하이젠알앤엠</t>
+  </si>
+  <si>
+    <t>한국제15호스팩</t>
+  </si>
+  <si>
+    <t>에스오에스랩</t>
+  </si>
+  <si>
+    <t>미래에셋비전스팩6호</t>
+  </si>
+  <si>
+    <t>KB제29호스팩</t>
+  </si>
+  <si>
+    <t>에이치엠씨제7호스팩</t>
+  </si>
+  <si>
+    <t>신한글로벌액티브리츠</t>
+  </si>
+  <si>
+    <t>코스닥</t>
+  </si>
+  <si>
+    <t>코스피</t>
+  </si>
+  <si>
+    <t>미래</t>
+  </si>
+  <si>
+    <t>삼성</t>
+  </si>
+  <si>
+    <t>키움</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>대신</t>
+  </si>
+  <si>
+    <t>한국</t>
+  </si>
+  <si>
+    <t>제이피모간회사</t>
+  </si>
+  <si>
+    <t>신한</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>BNK</t>
+  </si>
+  <si>
+    <t>KB</t>
+  </si>
+  <si>
+    <t>현대차</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>대표</t>
+  </si>
+  <si>
+    <t>인수</t>
+  </si>
+  <si>
+    <t>공동대표</t>
+  </si>
+  <si>
+    <t>2024-08-01</t>
+  </si>
+  <si>
+    <t>2024-07-22</t>
+  </si>
+  <si>
+    <t>2024-07-18</t>
+  </si>
+  <si>
+    <t>2024-07-16</t>
+  </si>
+  <si>
+    <t>2024-06-20</t>
+  </si>
+  <si>
     <t>2024-06-19</t>
   </si>
   <si>
-    <t>2024-07-01</t>
-  </si>
-  <si>
-    <t>아이빔테크놀로지</t>
-  </si>
-  <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
-    <t>산일전기</t>
-  </si>
-  <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
-    <t>SK증권제13호스팩</t>
-  </si>
-  <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
-    <t>시프트업</t>
-  </si>
-  <si>
-    <t>이베스트스팩6호</t>
-  </si>
-  <si>
-    <t>하스</t>
-  </si>
-  <si>
-    <t>이노스페이스</t>
-  </si>
-  <si>
-    <t>에이치브이엠</t>
-  </si>
-  <si>
-    <t>하이젠알앤엠</t>
-  </si>
-  <si>
-    <t>한국제15호스팩</t>
-  </si>
-  <si>
-    <t>에스오에스랩</t>
-  </si>
-  <si>
-    <t>미래에셋비전스팩6호</t>
-  </si>
-  <si>
-    <t>KB제29호스팩</t>
-  </si>
-  <si>
-    <t>에이치엠씨제7호스팩</t>
-  </si>
-  <si>
-    <t>한국제14호스팩</t>
-  </si>
-  <si>
-    <t>미래에셋비전스팩5호</t>
-  </si>
-  <si>
-    <t>씨어스테크놀로지</t>
-  </si>
-  <si>
-    <t>한중엔시에스</t>
-  </si>
-  <si>
-    <t>신한글로벌액티브리츠</t>
-  </si>
-  <si>
-    <t>코스닥</t>
-  </si>
-  <si>
-    <t>코스피</t>
-  </si>
-  <si>
-    <t>삼성</t>
-  </si>
-  <si>
-    <t>키움</t>
-  </si>
-  <si>
-    <t>미래</t>
-  </si>
-  <si>
-    <t>NH</t>
-  </si>
-  <si>
-    <t>SK</t>
-  </si>
-  <si>
-    <t>대신</t>
-  </si>
-  <si>
-    <t>한국</t>
-  </si>
-  <si>
-    <t>제이피모간회사</t>
-  </si>
-  <si>
-    <t>신한</t>
-  </si>
-  <si>
-    <t>LS</t>
-  </si>
-  <si>
-    <t>BNK</t>
-  </si>
-  <si>
-    <t>KB</t>
-  </si>
-  <si>
-    <t>현대차</t>
-  </si>
-  <si>
-    <t>IBK</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>대표</t>
-  </si>
-  <si>
-    <t>인수</t>
-  </si>
-  <si>
-    <t>공동대표</t>
-  </si>
-  <si>
-    <t>2024-07-22</t>
-  </si>
-  <si>
-    <t>2024-07-18</t>
-  </si>
-  <si>
-    <t>2024-07-16</t>
-  </si>
-  <si>
-    <t>2024-06-20</t>
-  </si>
-  <si>
     <t>2024-06-18</t>
   </si>
   <si>
@@ -272,9 +266,6 @@
   </si>
   <si>
     <t>2024-06-11</t>
-  </si>
-  <si>
-    <t>2024-06-10</t>
   </si>
   <si>
     <t>2024-07-30</t>
@@ -647,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -711,49 +702,49 @@
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D2">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F2">
-        <v>223.4</v>
+        <v>224</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M2">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N2">
         <v>100</v>
       </c>
       <c r="O2" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="P2" t="s">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="Q2">
-        <v>1675500</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -764,49 +755,49 @@
         <v>36</v>
       </c>
       <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3">
+        <v>223.4</v>
+      </c>
+      <c r="E3" t="s">
         <v>57</v>
       </c>
-      <c r="D3">
-        <v>297</v>
-      </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
       <c r="F3">
-        <v>297</v>
+        <v>223.4</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M3">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N3">
         <v>100</v>
       </c>
       <c r="O3" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="P3" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="Q3">
-        <v>1012500</v>
+        <v>1675500</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -817,99 +808,99 @@
         <v>37</v>
       </c>
       <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4">
+        <v>297</v>
+      </c>
+      <c r="E4" t="s">
         <v>58</v>
       </c>
-      <c r="D4">
-        <v>2660</v>
-      </c>
-      <c r="E4" t="s">
-        <v>61</v>
-      </c>
       <c r="F4">
-        <v>2553.6</v>
+        <v>297</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K4" t="s">
+        <v>70</v>
+      </c>
+      <c r="L4" t="s">
+        <v>69</v>
+      </c>
+      <c r="M4">
+        <v>22000</v>
+      </c>
+      <c r="N4">
+        <v>100</v>
+      </c>
+      <c r="O4" t="s">
         <v>74</v>
       </c>
-      <c r="L4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M4">
-        <v>35000</v>
-      </c>
-      <c r="N4">
-        <v>96</v>
-      </c>
-      <c r="O4" t="s">
-        <v>78</v>
-      </c>
       <c r="P4" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="Q4">
-        <v>9340690</v>
+        <v>1012500</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D5">
         <v>2660</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F5">
-        <v>106.4</v>
+        <v>2553.6</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="L5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M5">
         <v>35000</v>
       </c>
       <c r="N5">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="O5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="P5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Q5">
         <v>9340690</v>
@@ -923,49 +914,49 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6">
+        <v>2660</v>
+      </c>
+      <c r="E6" t="s">
         <v>57</v>
       </c>
-      <c r="D6">
-        <v>120</v>
-      </c>
-      <c r="E6" t="s">
-        <v>62</v>
-      </c>
       <c r="F6">
-        <v>120</v>
+        <v>106.4</v>
       </c>
       <c r="G6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M6">
-        <v>2000</v>
+        <v>35000</v>
       </c>
       <c r="N6">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O6" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="P6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="Q6">
-        <v>4500000</v>
+        <v>9340690</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -976,34 +967,34 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D7">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F7">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M7">
         <v>2000</v>
@@ -1012,13 +1003,13 @@
         <v>100</v>
       </c>
       <c r="O7" t="s">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="P7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="Q7">
-        <v>3000000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1029,49 +1020,49 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D8">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F8">
-        <v>161.8</v>
+        <v>80</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M8">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N8">
         <v>100</v>
       </c>
       <c r="O8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P8" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="Q8">
-        <v>1187900</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1082,87 +1073,87 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D9">
-        <v>4350</v>
+        <v>161.8</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F9">
-        <v>1435.5</v>
+        <v>161.8</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M9">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="N9">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O9" t="s">
         <v>26</v>
       </c>
       <c r="P9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="Q9">
-        <v>21750000</v>
+        <v>1187900</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D10">
         <v>4350</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F10">
         <v>1435.5</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K10" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M10">
         <v>60000</v>
@@ -1171,10 +1162,10 @@
         <v>33</v>
       </c>
       <c r="O10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Q10">
         <v>21750000</v>
@@ -1182,52 +1173,52 @@
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D11">
         <v>4350</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F11">
-        <v>1305</v>
+        <v>1435.5</v>
       </c>
       <c r="G11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K11" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M11">
         <v>60000</v>
       </c>
       <c r="N11">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Q11">
         <v>21750000</v>
@@ -1235,52 +1226,52 @@
     </row>
     <row r="12" spans="1:17">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D12">
         <v>4350</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F12">
-        <v>174</v>
+        <v>1305</v>
       </c>
       <c r="G12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="L12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M12">
         <v>60000</v>
       </c>
       <c r="N12">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="O12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Q12">
         <v>21750000</v>
@@ -1294,49 +1285,49 @@
         <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D13">
-        <v>80</v>
+        <v>4350</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F13">
-        <v>80</v>
+        <v>174</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K13" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M13">
-        <v>2000</v>
+        <v>60000</v>
       </c>
       <c r="N13">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="O13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Q13">
-        <v>3000000</v>
+        <v>21750000</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1347,49 +1338,49 @@
         <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D14">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F14">
-        <v>289.6</v>
+        <v>80</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K14" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M14">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N14">
         <v>100</v>
       </c>
       <c r="O14" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="P14" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="Q14">
-        <v>1357500</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1400,99 +1391,99 @@
         <v>44</v>
       </c>
       <c r="C15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15">
+        <v>289.6</v>
+      </c>
+      <c r="E15" t="s">
         <v>57</v>
       </c>
-      <c r="D15">
-        <v>575.89</v>
-      </c>
-      <c r="E15" t="s">
-        <v>61</v>
-      </c>
       <c r="F15">
-        <v>541.3366</v>
+        <v>289.6</v>
       </c>
       <c r="G15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M15">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="N15">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="O15" t="s">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="P15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q15">
-        <v>1906400</v>
+        <v>1357500</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D16">
         <v>575.89</v>
       </c>
       <c r="E16" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F16">
-        <v>34.5534</v>
+        <v>541.3366</v>
       </c>
       <c r="G16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K16" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="L16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M16">
         <v>43300</v>
       </c>
       <c r="N16">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="O16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="P16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q16">
         <v>1906400</v>
@@ -1506,49 +1497,49 @@
         <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D17">
-        <v>432</v>
+        <v>575.89</v>
       </c>
       <c r="E17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F17">
-        <v>432</v>
+        <v>34.5534</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K17" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L17" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M17">
-        <v>18000</v>
+        <v>43300</v>
       </c>
       <c r="N17">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="O17" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="P17" t="s">
         <v>31</v>
       </c>
       <c r="Q17">
-        <v>1758600</v>
+        <v>1906400</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1559,49 +1550,49 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D18">
-        <v>238</v>
+        <v>432</v>
       </c>
       <c r="E18" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F18">
-        <v>238</v>
+        <v>432</v>
       </c>
       <c r="G18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K18" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M18">
-        <v>7000</v>
+        <v>18000</v>
       </c>
       <c r="N18">
         <v>100</v>
       </c>
       <c r="O18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="P18" t="s">
         <v>32</v>
       </c>
       <c r="Q18">
-        <v>2350000</v>
+        <v>1758600</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1612,49 +1603,49 @@
         <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D19">
-        <v>125</v>
+        <v>238</v>
       </c>
       <c r="E19" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F19">
-        <v>125</v>
+        <v>238</v>
       </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K19" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L19" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M19">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N19">
         <v>100</v>
       </c>
       <c r="O19" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="P19" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="Q19">
-        <v>4687500</v>
+        <v>2350000</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1665,99 +1656,99 @@
         <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D20">
-        <v>230</v>
+        <v>125</v>
       </c>
       <c r="E20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F20">
-        <v>218.5</v>
+        <v>125</v>
       </c>
       <c r="G20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M20">
-        <v>11500</v>
+        <v>2000</v>
       </c>
       <c r="N20">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="O20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="P20" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="Q20">
-        <v>3000000</v>
+        <v>4687500</v>
       </c>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D21">
         <v>230</v>
       </c>
       <c r="E21" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F21">
-        <v>11.5</v>
+        <v>218.5</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K21" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="L21" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M21">
         <v>11500</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="O21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="P21" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="Q21">
         <v>3000000</v>
@@ -1771,49 +1762,49 @@
         <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D22">
-        <v>129</v>
+        <v>230</v>
       </c>
       <c r="E22" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F22">
-        <v>129</v>
+        <v>11.5</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M22">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="N22">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="O22" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="P22" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="Q22">
-        <v>4837500</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -1824,34 +1815,34 @@
         <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D23">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="E23" t="s">
+        <v>56</v>
+      </c>
+      <c r="F23">
+        <v>129</v>
+      </c>
+      <c r="G23" t="s">
+        <v>69</v>
+      </c>
+      <c r="H23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I23" t="s">
+        <v>69</v>
+      </c>
+      <c r="J23" t="s">
+        <v>69</v>
+      </c>
+      <c r="K23" t="s">
         <v>70</v>
       </c>
-      <c r="F23">
-        <v>120</v>
-      </c>
-      <c r="G23" t="s">
-        <v>73</v>
-      </c>
-      <c r="H23" t="s">
-        <v>73</v>
-      </c>
-      <c r="I23" t="s">
-        <v>73</v>
-      </c>
-      <c r="J23" t="s">
-        <v>73</v>
-      </c>
-      <c r="K23" t="s">
-        <v>74</v>
-      </c>
       <c r="L23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M23">
         <v>2000</v>
@@ -1860,51 +1851,51 @@
         <v>100</v>
       </c>
       <c r="O23" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="P23" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="Q23">
-        <v>4500000</v>
+        <v>4837500</v>
       </c>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B24" t="s">
         <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D24">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="E24" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F24">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K24" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M24">
         <v>2000</v>
@@ -1913,51 +1904,51 @@
         <v>100</v>
       </c>
       <c r="O24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="P24" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="Q24">
-        <v>5250000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="25" spans="1:17">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
         <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D25">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="E25" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F25">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K25" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L25" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M25">
         <v>2000</v>
@@ -1966,277 +1957,118 @@
         <v>100</v>
       </c>
       <c r="O25" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="P25" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="Q25">
-        <v>3000000</v>
+        <v>5250000</v>
       </c>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B26" t="s">
         <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D26">
-        <v>95</v>
+        <v>700.0000199999999</v>
       </c>
       <c r="E26" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F26">
-        <v>95</v>
+        <v>350.00001</v>
       </c>
       <c r="G26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M26">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="N26">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O26" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="P26" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Q26">
-        <v>3562500</v>
+        <v>32666668</v>
       </c>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D27">
-        <v>221</v>
+        <v>700.0000199999999</v>
       </c>
       <c r="E27" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F27">
-        <v>221</v>
+        <v>350.00001</v>
       </c>
       <c r="G27" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H27" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I27" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J27" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K27" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L27" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M27">
-        <v>17000</v>
+        <v>3000</v>
       </c>
       <c r="N27">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O27" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="P27" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Q27">
-        <v>975000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17">
-      <c r="A28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" t="s">
-        <v>57</v>
-      </c>
-      <c r="D28">
-        <v>480</v>
-      </c>
-      <c r="E28" t="s">
-        <v>72</v>
-      </c>
-      <c r="F28">
-        <v>480</v>
-      </c>
-      <c r="G28" t="s">
-        <v>73</v>
-      </c>
-      <c r="H28" t="s">
-        <v>73</v>
-      </c>
-      <c r="I28" t="s">
-        <v>73</v>
-      </c>
-      <c r="J28" t="s">
-        <v>73</v>
-      </c>
-      <c r="K28" t="s">
-        <v>74</v>
-      </c>
-      <c r="L28" t="s">
-        <v>73</v>
-      </c>
-      <c r="M28">
-        <v>30000</v>
-      </c>
-      <c r="N28">
-        <v>100</v>
-      </c>
-      <c r="O28" t="s">
-        <v>86</v>
-      </c>
-      <c r="P28" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q28">
-        <v>1123925</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17">
-      <c r="A29" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" t="s">
-        <v>58</v>
-      </c>
-      <c r="D29">
-        <v>700.0000199999999</v>
-      </c>
-      <c r="E29" t="s">
-        <v>67</v>
-      </c>
-      <c r="F29">
-        <v>350.00001</v>
-      </c>
-      <c r="G29" t="s">
-        <v>73</v>
-      </c>
-      <c r="H29" t="s">
-        <v>73</v>
-      </c>
-      <c r="I29" t="s">
-        <v>73</v>
-      </c>
-      <c r="J29" t="s">
-        <v>73</v>
-      </c>
-      <c r="K29" t="s">
-        <v>76</v>
-      </c>
-      <c r="L29" t="s">
-        <v>73</v>
-      </c>
-      <c r="M29">
-        <v>3000</v>
-      </c>
-      <c r="N29">
-        <v>50</v>
-      </c>
-      <c r="O29" t="s">
-        <v>84</v>
-      </c>
-      <c r="P29" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q29">
-        <v>32666668</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17">
-      <c r="A30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30" t="s">
-        <v>58</v>
-      </c>
-      <c r="D30">
-        <v>700.0000199999999</v>
-      </c>
-      <c r="E30" t="s">
-        <v>65</v>
-      </c>
-      <c r="F30">
-        <v>350.00001</v>
-      </c>
-      <c r="G30" t="s">
-        <v>73</v>
-      </c>
-      <c r="H30" t="s">
-        <v>73</v>
-      </c>
-      <c r="I30" t="s">
-        <v>73</v>
-      </c>
-      <c r="J30" t="s">
-        <v>73</v>
-      </c>
-      <c r="K30" t="s">
-        <v>76</v>
-      </c>
-      <c r="L30" t="s">
-        <v>73</v>
-      </c>
-      <c r="M30">
-        <v>3000</v>
-      </c>
-      <c r="N30">
-        <v>50</v>
-      </c>
-      <c r="O30" t="s">
-        <v>84</v>
-      </c>
-      <c r="P30" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q30">
         <v>32666668</v>
       </c>
     </row>

</xml_diff>